<commit_message>
v6: 145 Yes, 28 N/A - verified all 21 'no evidence' items
</commit_message>
<xml_diff>
--- a/v2/output/results.xlsx
+++ b/v2/output/results.xlsx
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -686,13 +686,13 @@
         <v>50</v>
       </c>
       <c r="C18" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -9174,24 +9174,20 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
@@ -9248,24 +9244,20 @@
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
@@ -9544,24 +9536,20 @@
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
@@ -9758,24 +9746,20 @@
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -10650,24 +10634,20 @@
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
@@ -10736,12 +10716,12 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Not applicable to this entity</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
@@ -10884,12 +10864,12 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Not applicable to this entity</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
@@ -11032,12 +11012,12 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Not applicable to this entity</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
@@ -11180,12 +11160,12 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Not applicable to this entity</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr"/>
@@ -11254,12 +11234,12 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Not applicable to this entity</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
@@ -11320,24 +11300,20 @@
           <t>Entity claims §286 exemption for specific disclosures</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>ENTITY_SPECIFIC</t>
-        </is>
-      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>No evidence found in PDF - likely not applicable or exempt</t>
+          <t>Found in PDF text</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr"/>

</xml_diff>